<commit_message>
Add Continuous Monitoring Dashboard tab and AAC Access Model config guide
</commit_message>
<xml_diff>
--- a/grc-workpapers/GRC_ITAC_Audit_Workpaper_Package.xlsx
+++ b/grc-workpapers/GRC_ITAC_Audit_Workpaper_Package.xlsx
@@ -26,7 +26,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Deficiency_Log" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Remediation_Roadmap" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_Findings_Report" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19_Sampling_Guidance" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19_Monitoring_Dashboard" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20_Sampling_Guidance" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -166,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -214,6 +215,21 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -581,7 +597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E28"/>
+  <dimension ref="B2:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -1032,29 +1048,51 @@
     <row r="25">
       <c r="B25" s="4" t="inlineStr">
         <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Monitoring</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>19_Monitoring_Dashboard</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Continuous monitoring KPIs &amp; metrics</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="5" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>19_Sampling_Guidance</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>20_Sampling_Guidance</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>Sample size reference &amp; tickmark legend</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Companion Word deliverables: Scoping_Memorandum.docx, Findings_Report.docx (see grc-workpapers folder).</t>
+    <row r="29">
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Companion Word deliverables: Scoping_Memorandum.docx, Findings_Report.docx, AAC_Access_Model_Config_Guide.docx (see grc-workpapers folder).</t>
         </is>
       </c>
     </row>
@@ -7395,6 +7433,889 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F6E43"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:G56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>CONTINUOUS MONITORING DASHBOARD - AAC / ATC METRICS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Near-real-time KPIs from Oracle AAC/ATC continuous monitoring. Population scanned: 342 users, 9,655 transactions. Refresh: with each data sync.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>1. HEADLINE KPIs</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Prior Period</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Total SoD incidents (open)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>64</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>78</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>&lt; 40</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>Off Track</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>New incidents this period</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Decreasing</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>On Track</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Incidents closed this period</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Increasing</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>On Track</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Critical incidents open</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>Off Track</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>High incidents open</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>&lt; 20</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>Off Track</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Avg age of open incidents (days)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>&lt; 30</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Mean time to remediate (days)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>&lt; 21</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>% incidents with mitigating control</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>72%</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>&gt; 90%</t>
+        </is>
+      </c>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>False positive rate</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>11%</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>24%</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>&lt; 10%</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Control coverage (processes w/ active controls)</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>70%</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Users with conflicts / total users</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>64 / 342 (19%)</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>78 / 340 (23%)</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>&lt; 10%</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>Off Track</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Overdue remediations</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>Off Track</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>2. INCIDENTS BY SEVERITY (status breakdown)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>In Investigation</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Remediate</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="23" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C23" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="20">
+        <f>SUM(C23:F23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="n">
+        <v>24</v>
+      </c>
+      <c r="D24" s="25" t="n">
+        <v>12</v>
+      </c>
+      <c r="E24" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="F24" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" s="25">
+        <f>SUM(C24:F24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="26" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C25" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="D25" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="E25" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F25" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="G25" s="20">
+        <f>SUM(C25:F25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="27" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C26" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="G26" s="25">
+        <f>SUM(C26:F26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>3. INCIDENTS BY PROCESS</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t># Incidents</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>% of Total</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Top Rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>P2P (Procure-to-Pay)</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>36%</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>SOD-03 (PO entry/approval)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>R2R (Record-to-Report)</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>22%</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>SOD-28 (JE create/approve)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>O2C (Order-to-Cash)</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>SOD-20 (credit memo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Payroll</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>12%</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>SOD-38 (ghost employee)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Security / Admin</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>SOD-73 (user admin)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>6%</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Various</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>4. OPEN INCIDENT AGING</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Age Bucket</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>SLA Breached?</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>0 - 30 days</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>31 - 60 days</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>61 - 90 days</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D43" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>90+ days</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D44" s="11" t="inlineStr">
+        <is>
+          <t>Yes - escalate</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>5. ATC TRANSACTION MONITORING (this period)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Txns Flagged</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed Issues</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Value at Risk (INR)</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>ATC-01 Duplicate Payments</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D49" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>8,40,000</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>Under Recovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>ATC-02 Ghost Vendor (bank match)</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D50" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>12,00,000</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>Investigating</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>ATC-12 Post-Termination Payments</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D51" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>2,15,000</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>Recovered</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>ATC-09 Large Manual Journals</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="D52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>Reviewed - OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>ATC-05 Split Transactions</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="D53" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>1,90,000</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>Investigating</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="15" t="inlineStr">
+        <is>
+          <t>Note: Metrics illustrate a monthly monitoring cadence. Green=on track, Amber=watch, Red=off track/breach.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00A6A6A6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -7564,7 +8485,7 @@
           <t>Y / tick</t>
         </is>
       </c>
-      <c r="C15" s="23" t="inlineStr">
+      <c r="C15" s="28" t="inlineStr">
         <is>
           <t>Verified to supporting evidence</t>
         </is>
@@ -7576,7 +8497,7 @@
           <t>N / cross</t>
         </is>
       </c>
-      <c r="C16" s="23" t="inlineStr">
+      <c r="C16" s="28" t="inlineStr">
         <is>
           <t>Exception noted</t>
         </is>
@@ -7588,7 +8509,7 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="C17" s="23" t="inlineStr">
+      <c r="C17" s="28" t="inlineStr">
         <is>
           <t>Attribute met, no exception</t>
         </is>
@@ -7600,7 +8521,7 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="C18" s="23" t="inlineStr">
+      <c r="C18" s="28" t="inlineStr">
         <is>
           <t>Attribute not met - deficiency</t>
         </is>
@@ -7612,7 +8533,7 @@
           <t>E</t>
         </is>
       </c>
-      <c r="C19" s="23" t="inlineStr">
+      <c r="C19" s="28" t="inlineStr">
         <is>
           <t>Evidence attached (referenced)</t>
         </is>
@@ -7624,7 +8545,7 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="C20" s="23" t="inlineStr">
+      <c r="C20" s="28" t="inlineStr">
         <is>
           <t>Not applicable</t>
         </is>

</xml_diff>